<commit_message>
feat: ajustes en dashboard y limpieza de archivos temporales
</commit_message>
<xml_diff>
--- a/data/kpis.xlsx
+++ b/data/kpis.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="60">
   <si>
     <t xml:space="preserve">Área</t>
   </si>
@@ -99,7 +99,7 @@
     <t xml:space="preserve">Azure DevOps / Jira</t>
   </si>
   <si>
-    <t xml:space="preserve">Ger. Desarrollo Software</t>
+    <t xml:space="preserve">Gobierno TI</t>
   </si>
   <si>
     <t xml:space="preserve">KPI-AE-02</t>
@@ -132,13 +132,10 @@
     <t xml:space="preserve">GitHub Copilot Telemetry</t>
   </si>
   <si>
-    <t xml:space="preserve">Ger. Transformación</t>
-  </si>
-  <si>
     <t xml:space="preserve">OTI04</t>
   </si>
   <si>
-    <t xml:space="preserve">Arquitectura Escalable y Modular</t>
+    <t xml:space="preserve">OTI4 – Arquitectura Escalable y Modular</t>
   </si>
   <si>
     <t xml:space="preserve">KPI-SW-08</t>
@@ -151,9 +148,6 @@
   </si>
   <si>
     <t xml:space="preserve">Architecture Review Board</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ger. Arquitectura SW</t>
   </si>
   <si>
     <t xml:space="preserve">KPI-SW-09</t>
@@ -502,9 +496,9 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="37.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="37.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="37.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="37.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.01"/>
@@ -645,7 +639,7 @@
       <c r="J3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L3" s="7" t="n">
@@ -696,7 +690,7 @@
         <v>35</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="L4" s="3" t="n">
         <v>0</v>
@@ -722,16 +716,16 @@
         <v>17</v>
       </c>
       <c r="C5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="8" t="s">
         <v>39</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>40</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>33</v>
@@ -740,13 +734,13 @@
         <v>60</v>
       </c>
       <c r="I5" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>43</v>
+      <c r="K5" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
@@ -762,16 +756,16 @@
         <v>17</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="E6" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>33</v>
@@ -780,13 +774,13 @@
         <v>70</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
@@ -796,52 +790,52 @@
     </row>
     <row r="7" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>51</v>
-      </c>
       <c r="E7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="N7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="P7" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -952,7 +946,7 @@
     </row>
     <row r="5" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0</v>
@@ -972,7 +966,7 @@
     </row>
     <row r="6" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>0</v>
@@ -1024,13 +1018,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
@@ -1047,10 +1041,10 @@
         <v>16</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>18</v>
@@ -1067,36 +1061,36 @@
         <v>16</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C4" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="12" t="s">
         <v>59</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>